<commit_message>
adjust colors of diagrams to fit to new ase.tools website
</commit_message>
<xml_diff>
--- a/docs/operation-modes.xlsx
+++ b/docs/operation-modes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rse/Work/ase/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE342786-BD43-AC49-A7C6-B5B03CDACA46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE888038-2182-D744-B00E-07A7FCBF1233}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11060" yWindow="7040" windowWidth="28040" windowHeight="17180" xr2:uid="{10B8B807-6256-AB4F-8C12-E23F0A365D36}"/>
   </bookViews>
@@ -125,7 +125,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -164,30 +164,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF5DBC1"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEBB57D"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDF8F37"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFB26813"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -198,8 +174,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1067B2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -219,21 +201,6 @@
       </top>
       <bottom style="thin">
         <color theme="1" tint="0.34998626667073579"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF71420D"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF71420D"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF71420D"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF71420D"/>
       </bottom>
       <diagonal/>
     </border>
@@ -301,37 +268,37 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -341,15 +308,15 @@
   <colors>
     <mruColors>
       <color rgb="FF0C4171"/>
+      <color rgb="FF1067B2"/>
+      <color rgb="FF368DDF"/>
+      <color rgb="FF7DB4EA"/>
+      <color rgb="FFC0DBF5"/>
       <color rgb="FF71420D"/>
       <color rgb="FFB26813"/>
       <color rgb="FFDF8F37"/>
       <color rgb="FFEBB57D"/>
       <color rgb="FFF5DBC1"/>
-      <color rgb="FF929292"/>
-      <color rgb="FF368DDF"/>
-      <color rgb="FF7DB4EA"/>
-      <color rgb="FFC0DBF5"/>
     </mruColors>
   </colors>
   <extLst>
@@ -695,36 +662,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" ht="145" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="F2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="11" t="s">
         <v>11</v>
       </c>
       <c r="I2" s="1"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
       <c r="G3" s="3"/>
       <c r="H3"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="13" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="4"/>
@@ -735,7 +702,7 @@
       <c r="H4"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="13" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="4"/>
@@ -746,7 +713,7 @@
       <c r="H5"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="14" t="s">
         <v>8</v>
       </c>
       <c r="C6" s="4"/>
@@ -757,7 +724,7 @@
       <c r="H6"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="14" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="4"/>
@@ -768,7 +735,7 @@
       <c r="H7"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="15" t="s">
         <v>10</v>
       </c>
       <c r="C8" s="4"/>
@@ -779,7 +746,7 @@
       <c r="H8"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="15" t="s">
         <v>9</v>
       </c>
       <c r="C9" s="4"/>

</xml_diff>